<commit_message>
fix(purchases): remove invalid empty string cells from Excel template
</commit_message>
<xml_diff>
--- a/public/templates/massar-purchase-template.xlsx
+++ b/public/templates/massar-purchase-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="البنود" sheetId="1" r:id="R3a400204a45941d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات وأمثلة" sheetId="2" r:id="Rbf629329ed634b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="البنود" sheetId="1" r:id="Rfd6529fc551f47f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات وأمثلة" sheetId="2" r:id="R45b2d62b5341463d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51,146 +51,44 @@
   <x:borders count="40">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1114,19 +1012,19 @@
       <x:c r="A1" s="108" t="str">
         <x:v>تعليمات تعبئة قالب فاتورة المشتريات</x:v>
       </x:c>
-      <x:c r="B1" s="62" t="str"/>
-      <x:c r="C1" s="62" t="str"/>
-      <x:c r="D1" s="62" t="str"/>
-      <x:c r="E1" s="62" t="str"/>
-      <x:c r="F1" s="62" t="str"/>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="62" t="str"/>
-      <x:c r="B2" s="62" t="str"/>
-      <x:c r="C2" s="62" t="str"/>
-      <x:c r="D2" s="62" t="str"/>
-      <x:c r="E2" s="62" t="str"/>
-      <x:c r="F2" s="62" t="str"/>
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="64" t="str">
@@ -1141,8 +1039,8 @@
       <x:c r="D3" s="66" t="str">
         <x:v>مثال</x:v>
       </x:c>
-      <x:c r="E3" s="62" t="str"/>
-      <x:c r="F3" s="62" t="str"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="67" t="str">
@@ -1157,8 +1055,8 @@
       <x:c r="D4" s="68" t="str">
         <x:v>كابل شحن Type-C</x:v>
       </x:c>
-      <x:c r="E4" s="62" t="str"/>
-      <x:c r="F4" s="62" t="str"/>
+      <x:c r="E4"/>
+      <x:c r="F4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="67" t="str">
@@ -1173,8 +1071,8 @@
       <x:c r="D5" s="68" t="str">
         <x:v>0012345678901</x:v>
       </x:c>
-      <x:c r="E5" s="62" t="str"/>
-      <x:c r="F5" s="62" t="str"/>
+      <x:c r="E5"/>
+      <x:c r="F5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="67" t="str">
@@ -1189,8 +1087,8 @@
       <x:c r="D6" s="68" t="str">
         <x:v>إكسسوارات</x:v>
       </x:c>
-      <x:c r="E6" s="62" t="str"/>
-      <x:c r="F6" s="62" t="str"/>
+      <x:c r="E6"/>
+      <x:c r="F6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="67" t="str">
@@ -1205,8 +1103,8 @@
       <x:c r="D7" s="68" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E7" s="62" t="str"/>
-      <x:c r="F7" s="62" t="str"/>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="67" t="str">
@@ -1221,8 +1119,8 @@
       <x:c r="D8" s="68" t="str">
         <x:v>12.50</x:v>
       </x:c>
-      <x:c r="E8" s="62" t="str"/>
-      <x:c r="F8" s="62" t="str"/>
+      <x:c r="E8"/>
+      <x:c r="F8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="69" t="str">
@@ -1237,18 +1135,18 @@
       <x:c r="D9" s="71" t="str">
         <x:v>20.00</x:v>
       </x:c>
-      <x:c r="E9" s="62" t="str"/>
-      <x:c r="F9" s="62" t="str"/>
+      <x:c r="E9"/>
+      <x:c r="F9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="62" t="str">
         <x:v>مثال تعبئة</x:v>
       </x:c>
-      <x:c r="B10" s="62" t="str"/>
-      <x:c r="C10" s="62" t="str"/>
-      <x:c r="D10" s="62" t="str"/>
-      <x:c r="E10" s="62" t="str"/>
-      <x:c r="F10" s="62" t="str"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="85" t="str">

</xml_diff>